<commit_message>
v10 core: allocator, constructs loader, genetic backgrounds, fish line loader
</commit_message>
<xml_diff>
--- a/seed_kits/2025-11-15-121231-autoload/fish.xlsx
+++ b/seed_kits/2025-11-15-121231-autoload/fish.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11116"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/davekokel/Projects/carp_v2/carp_app/seed_kits/fish/2025-11-05-fish/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/davekokel/Projects/carp_v2/seed_kits/2025-11-15-121231-autoload/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{010BB879-D7D0-734F-9438-9321ECAA1E9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2A6C7D9-BDB2-7441-9D38-94CCBB9CBA6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="18820" yWindow="7560" windowWidth="27640" windowHeight="24440" xr2:uid="{511D1851-48B7-274E-B5E4-033AFB6626E7}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="833" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="832" uniqueCount="114">
   <si>
     <t>membrane tandem mSG (ef1a:2xLynk:tdmStayGold)</t>
   </si>
@@ -828,7 +828,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D2D25443-873B-0B4C-9F55-D885A78791A6}">
-  <dimension ref="A1:I1019"/>
+  <dimension ref="A1:I1018"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="74.33203125" customWidth="1"/>
@@ -4024,30 +4024,36 @@
     </row>
     <row r="116" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A116" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="B116" s="12">
-        <v>45712</v>
+        <v>45520</v>
       </c>
       <c r="C116" t="s">
         <v>69</v>
       </c>
       <c r="D116" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="E116" t="s">
-        <v>100</v>
+        <v>1</v>
+      </c>
+      <c r="F116">
+        <v>301</v>
       </c>
       <c r="G116" t="s">
         <v>74</v>
       </c>
+      <c r="H116" t="s">
+        <v>75</v>
+      </c>
       <c r="I116" t="s">
-        <v>77</v>
+        <v>103</v>
       </c>
     </row>
     <row r="117" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A117" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="B117" s="12">
         <v>45520</v>
@@ -4062,7 +4068,7 @@
         <v>1</v>
       </c>
       <c r="F117">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="G117" t="s">
         <v>74</v>
@@ -4071,27 +4077,27 @@
         <v>75</v>
       </c>
       <c r="I117" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
     </row>
     <row r="118" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A118" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B118" s="12">
-        <v>45520</v>
+        <v>45620</v>
       </c>
       <c r="C118" t="s">
         <v>69</v>
       </c>
       <c r="D118" t="s">
-        <v>102</v>
+        <v>5</v>
       </c>
       <c r="E118" t="s">
         <v>1</v>
       </c>
       <c r="F118">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="G118" t="s">
         <v>74</v>
@@ -4100,15 +4106,15 @@
         <v>75</v>
       </c>
       <c r="I118" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
     </row>
     <row r="119" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A119" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B119" s="12">
-        <v>45620</v>
+        <v>45621</v>
       </c>
       <c r="C119" t="s">
         <v>69</v>
@@ -4120,7 +4126,7 @@
         <v>1</v>
       </c>
       <c r="F119">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="G119" t="s">
         <v>74</v>
@@ -4134,22 +4140,22 @@
     </row>
     <row r="120" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A120" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B120" s="12">
-        <v>45621</v>
+        <v>45764</v>
       </c>
       <c r="C120" t="s">
         <v>69</v>
       </c>
       <c r="D120" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E120" t="s">
         <v>1</v>
       </c>
       <c r="F120">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="G120" t="s">
         <v>74</v>
@@ -4158,15 +4164,15 @@
         <v>75</v>
       </c>
       <c r="I120" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
     </row>
     <row r="121" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A121" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B121" s="12">
-        <v>45764</v>
+        <v>45719</v>
       </c>
       <c r="C121" t="s">
         <v>69</v>
@@ -4178,7 +4184,7 @@
         <v>1</v>
       </c>
       <c r="F121">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="G121" t="s">
         <v>74</v>
@@ -4192,51 +4198,42 @@
     </row>
     <row r="122" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A122" t="s">
-        <v>111</v>
+        <v>69</v>
       </c>
       <c r="B122" s="12">
-        <v>45719</v>
+        <v>45938</v>
       </c>
       <c r="C122" t="s">
         <v>69</v>
       </c>
       <c r="D122" t="s">
-        <v>6</v>
-      </c>
-      <c r="E122" t="s">
-        <v>1</v>
-      </c>
-      <c r="F122">
-        <v>302</v>
-      </c>
-      <c r="G122" t="s">
-        <v>74</v>
+        <v>99</v>
       </c>
       <c r="H122" t="s">
-        <v>75</v>
+        <v>112</v>
       </c>
       <c r="I122" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
     </row>
     <row r="123" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A123" t="s">
-        <v>69</v>
+        <v>98</v>
       </c>
       <c r="B123" s="12">
-        <v>45938</v>
+        <v>45712</v>
       </c>
       <c r="C123" t="s">
-        <v>69</v>
+        <v>100</v>
       </c>
       <c r="D123" t="s">
         <v>99</v>
       </c>
-      <c r="H123" t="s">
-        <v>112</v>
+      <c r="G123" t="s">
+        <v>74</v>
       </c>
       <c r="I123" t="s">
-        <v>113</v>
+        <v>77</v>
       </c>
     </row>
     <row r="124" spans="1:9" x14ac:dyDescent="0.2">
@@ -12291,20 +12288,11 @@
       <c r="C1018" s="1"/>
       <c r="D1018" s="1"/>
       <c r="E1018" s="1"/>
-      <c r="F1018" s="1"/>
       <c r="I1018" s="1"/>
     </row>
-    <row r="1019" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A1019" s="1"/>
-      <c r="B1019" s="1"/>
-      <c r="C1019" s="1"/>
-      <c r="D1019" s="1"/>
-      <c r="E1019" s="1"/>
-      <c r="I1019" s="1"/>
-    </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G1067">
-    <sortCondition ref="B2:B1067"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G1066">
+    <sortCondition ref="B2:B1066"/>
   </sortState>
   <phoneticPr fontId="11" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
v11 fish loader stack: instance-driven genotypes, backgrounds, and views
</commit_message>
<xml_diff>
--- a/seed_kits/2025-11-15-121231-autoload/fish.xlsx
+++ b/seed_kits/2025-11-15-121231-autoload/fish.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/davekokel/Projects/carp_v2/seed_kits/2025-11-15-121231-autoload/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2A6C7D9-BDB2-7441-9D38-94CCBB9CBA6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{961A187F-C9CD-B04D-BE86-24008DE285B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="18820" yWindow="7560" windowWidth="27640" windowHeight="24440" xr2:uid="{511D1851-48B7-274E-B5E4-033AFB6626E7}"/>
+    <workbookView xWindow="6920" yWindow="680" windowWidth="27640" windowHeight="19860" xr2:uid="{511D1851-48B7-274E-B5E4-033AFB6626E7}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -233,13 +233,7 @@
     <t>birthday</t>
   </si>
   <si>
-    <t>line_building_stage</t>
-  </si>
-  <si>
     <t>allele_nickname</t>
-  </si>
-  <si>
-    <t>nickname</t>
   </si>
   <si>
     <t>genetic_background</t>
@@ -378,6 +372,12 @@
   </si>
   <si>
     <t>test line</t>
+  </si>
+  <si>
+    <t>line_nickname</t>
+  </si>
+  <si>
+    <t>instance_stage</t>
   </si>
 </sst>
 </file>
@@ -840,28 +840,28 @@
   <sheetData>
     <row r="1" spans="1:9" ht="30" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
-        <v>67</v>
+        <v>112</v>
       </c>
       <c r="B1" t="s">
         <v>64</v>
       </c>
       <c r="C1" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="D1" t="s">
-        <v>65</v>
+        <v>113</v>
       </c>
       <c r="E1" t="s">
         <v>62</v>
       </c>
       <c r="F1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="G1" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="H1" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="I1" s="3" t="s">
         <v>63</v>
@@ -875,7 +875,7 @@
         <v>45512</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>3</v>
@@ -885,10 +885,10 @@
       </c>
       <c r="F2" s="1"/>
       <c r="G2" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H2" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I2" s="4" t="s">
         <v>2</v>
@@ -902,7 +902,7 @@
         <v>45520</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D3" s="4" t="s">
         <v>4</v>
@@ -914,10 +914,10 @@
         <v>301</v>
       </c>
       <c r="G3" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H3" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I3" s="4" t="s">
         <v>2</v>
@@ -931,7 +931,7 @@
         <v>45520</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D4" s="4" t="s">
         <v>4</v>
@@ -943,10 +943,10 @@
         <v>302</v>
       </c>
       <c r="G4" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H4" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I4" s="4" t="s">
         <v>2</v>
@@ -960,7 +960,7 @@
         <v>45520</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D5" s="4" t="s">
         <v>4</v>
@@ -972,10 +972,10 @@
         <v>303</v>
       </c>
       <c r="G5" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H5" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I5" s="4" t="s">
         <v>2</v>
@@ -989,7 +989,7 @@
         <v>45520</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D6" s="4" t="s">
         <v>4</v>
@@ -1001,10 +1001,10 @@
         <v>305</v>
       </c>
       <c r="G6" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H6" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I6" s="4" t="s">
         <v>2</v>
@@ -1018,7 +1018,7 @@
         <v>45520</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D7" s="4" t="s">
         <v>4</v>
@@ -1030,10 +1030,10 @@
         <v>305</v>
       </c>
       <c r="G7" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H7" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I7" s="4" t="s">
         <v>2</v>
@@ -1047,7 +1047,7 @@
         <v>45520</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D8" s="4" t="s">
         <v>4</v>
@@ -1059,10 +1059,10 @@
         <v>306</v>
       </c>
       <c r="G8" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H8" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I8" s="4" t="s">
         <v>2</v>
@@ -1076,22 +1076,22 @@
         <v>45525</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D9" s="4" t="s">
         <v>5</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="G9" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H9" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I9" s="4" t="s">
         <v>2</v>
@@ -1105,7 +1105,7 @@
         <v>45566</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D10" s="4" t="s">
         <v>3</v>
@@ -1115,10 +1115,10 @@
       </c>
       <c r="F10" s="1"/>
       <c r="G10" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H10" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I10" s="7" t="s">
         <v>2</v>
@@ -1132,7 +1132,7 @@
         <v>45566</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D11" s="4" t="s">
         <v>3</v>
@@ -1142,10 +1142,10 @@
       </c>
       <c r="F11" s="4"/>
       <c r="G11" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H11" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I11" s="7" t="s">
         <v>2</v>
@@ -1159,7 +1159,7 @@
         <v>45566</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D12" s="4" t="s">
         <v>4</v>
@@ -1171,10 +1171,10 @@
         <v>318</v>
       </c>
       <c r="G12" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H12" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I12" s="7" t="s">
         <v>2</v>
@@ -1188,7 +1188,7 @@
         <v>45566</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D13" s="4" t="s">
         <v>4</v>
@@ -1200,10 +1200,10 @@
         <v>319</v>
       </c>
       <c r="G13" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H13" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I13" s="7" t="s">
         <v>2</v>
@@ -1217,7 +1217,7 @@
         <v>45608</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D14" s="4" t="s">
         <v>5</v>
@@ -1229,10 +1229,10 @@
         <v>301</v>
       </c>
       <c r="G14" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H14" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I14" s="4" t="s">
         <v>2</v>
@@ -1246,7 +1246,7 @@
         <v>45616</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D15" s="4" t="s">
         <v>3</v>
@@ -1256,10 +1256,10 @@
       </c>
       <c r="F15" s="4"/>
       <c r="G15" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H15" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I15" s="7" t="s">
         <v>2</v>
@@ -1273,7 +1273,7 @@
         <v>45616</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D16" s="4" t="s">
         <v>4</v>
@@ -1285,10 +1285,10 @@
         <v>311</v>
       </c>
       <c r="G16" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H16" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I16" s="7" t="s">
         <v>2</v>
@@ -1302,7 +1302,7 @@
         <v>45616</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D17" s="4" t="s">
         <v>4</v>
@@ -1314,10 +1314,10 @@
         <v>312</v>
       </c>
       <c r="G17" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H17" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I17" s="7" t="s">
         <v>2</v>
@@ -1331,7 +1331,7 @@
         <v>45616</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D18" s="4" t="s">
         <v>4</v>
@@ -1343,10 +1343,10 @@
         <v>313</v>
       </c>
       <c r="G18" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H18" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I18" s="7" t="s">
         <v>2</v>
@@ -1360,7 +1360,7 @@
         <v>45616</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D19" s="4" t="s">
         <v>4</v>
@@ -1372,10 +1372,10 @@
         <v>314</v>
       </c>
       <c r="G19" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H19" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I19" s="7" t="s">
         <v>2</v>
@@ -1389,7 +1389,7 @@
         <v>45621</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D20" s="4" t="s">
         <v>5</v>
@@ -1401,10 +1401,10 @@
         <v>302</v>
       </c>
       <c r="G20" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H20" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I20" s="4" t="s">
         <v>2</v>
@@ -1418,7 +1418,7 @@
         <v>45621</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D21" s="4" t="s">
         <v>41</v>
@@ -1428,10 +1428,10 @@
       </c>
       <c r="F21" s="4"/>
       <c r="G21" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H21" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I21" s="8" t="s">
         <v>2</v>
@@ -1445,7 +1445,7 @@
         <v>45621</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D22" s="4" t="s">
         <v>4</v>
@@ -1457,10 +1457,10 @@
         <v>338</v>
       </c>
       <c r="G22" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H22" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I22" s="8" t="s">
         <v>2</v>
@@ -1474,7 +1474,7 @@
         <v>45631</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D23" s="4" t="s">
         <v>3</v>
@@ -1484,10 +1484,10 @@
       </c>
       <c r="F23" s="4"/>
       <c r="G23" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H23" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I23" s="6" t="s">
         <v>10</v>
@@ -1501,7 +1501,7 @@
         <v>45659</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D24" s="4" t="s">
         <v>3</v>
@@ -1511,10 +1511,10 @@
       </c>
       <c r="F24" s="1"/>
       <c r="G24" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H24" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I24" s="8" t="s">
         <v>2</v>
@@ -1528,7 +1528,7 @@
         <v>45664</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D25" s="4" t="s">
         <v>4</v>
@@ -1540,10 +1540,10 @@
         <v>339</v>
       </c>
       <c r="G25" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H25" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I25" s="8" t="s">
         <v>2</v>
@@ -1557,7 +1557,7 @@
         <v>45710</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D26" s="4" t="s">
         <v>3</v>
@@ -1567,10 +1567,10 @@
       </c>
       <c r="F26" s="4"/>
       <c r="G26" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H26" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I26" s="8" t="s">
         <v>2</v>
@@ -1584,7 +1584,7 @@
         <v>45710</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D27" s="4" t="s">
         <v>4</v>
@@ -1596,10 +1596,10 @@
         <v>322</v>
       </c>
       <c r="G27" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H27" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I27" s="8" t="s">
         <v>2</v>
@@ -1613,7 +1613,7 @@
         <v>45710</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D28" s="4" t="s">
         <v>4</v>
@@ -1625,10 +1625,10 @@
         <v>323</v>
       </c>
       <c r="G28" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H28" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I28" s="8" t="s">
         <v>2</v>
@@ -1642,7 +1642,7 @@
         <v>45713</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D29" s="4" t="s">
         <v>3</v>
@@ -1652,10 +1652,10 @@
       </c>
       <c r="F29" s="4"/>
       <c r="G29" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H29" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I29" s="7" t="s">
         <v>2</v>
@@ -1669,7 +1669,7 @@
         <v>45713</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D30" s="4" t="s">
         <v>4</v>
@@ -1681,10 +1681,10 @@
         <v>320</v>
       </c>
       <c r="G30" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H30" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I30" s="7" t="s">
         <v>2</v>
@@ -1698,7 +1698,7 @@
         <v>45713</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D31" s="4" t="s">
         <v>4</v>
@@ -1710,10 +1710,10 @@
         <v>321</v>
       </c>
       <c r="G31" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H31" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I31" s="7" t="s">
         <v>2</v>
@@ -1727,7 +1727,7 @@
         <v>45714</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D32" s="4" t="s">
         <v>4</v>
@@ -1739,10 +1739,10 @@
         <v>309</v>
       </c>
       <c r="G32" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H32" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I32" s="7" t="s">
         <v>2</v>
@@ -1756,7 +1756,7 @@
         <v>45714</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D33" s="4" t="s">
         <v>4</v>
@@ -1768,10 +1768,10 @@
         <v>310</v>
       </c>
       <c r="G33" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H33" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I33" s="7" t="s">
         <v>2</v>
@@ -1785,7 +1785,7 @@
         <v>45714</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D34" s="4" t="s">
         <v>5</v>
@@ -1797,10 +1797,10 @@
         <v>318</v>
       </c>
       <c r="G34" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H34" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I34" s="7" t="s">
         <v>2</v>
@@ -1814,7 +1814,7 @@
         <v>45714</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D35" s="4" t="s">
         <v>5</v>
@@ -1826,10 +1826,10 @@
         <v>319</v>
       </c>
       <c r="G35" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H35" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I35" s="7" t="s">
         <v>2</v>
@@ -1843,7 +1843,7 @@
         <v>45719</v>
       </c>
       <c r="C36" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D36" s="4" t="s">
         <v>6</v>
@@ -1855,10 +1855,10 @@
         <v>302</v>
       </c>
       <c r="G36" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H36" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I36" s="4" t="s">
         <v>2</v>
@@ -1872,7 +1872,7 @@
         <v>45749</v>
       </c>
       <c r="C37" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D37" s="4" t="s">
         <v>47</v>
@@ -1882,10 +1882,10 @@
       </c>
       <c r="F37" s="1"/>
       <c r="G37" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H37" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I37" s="8" t="s">
         <v>2</v>
@@ -1899,7 +1899,7 @@
         <v>45755</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D38" s="4" t="s">
         <v>4</v>
@@ -1911,10 +1911,10 @@
         <v>324</v>
       </c>
       <c r="G38" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H38" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I38" s="8" t="s">
         <v>2</v>
@@ -1928,7 +1928,7 @@
         <v>45762</v>
       </c>
       <c r="C39" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D39" s="4" t="s">
         <v>41</v>
@@ -1938,10 +1938,10 @@
       </c>
       <c r="F39" s="1"/>
       <c r="G39" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H39" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I39" s="8" t="s">
         <v>2</v>
@@ -1955,7 +1955,7 @@
         <v>45763</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D40" s="4" t="s">
         <v>3</v>
@@ -1965,10 +1965,10 @@
       </c>
       <c r="F40" s="4"/>
       <c r="G40" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H40" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I40" s="6" t="s">
         <v>2</v>
@@ -1982,7 +1982,7 @@
         <v>45763</v>
       </c>
       <c r="C41" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D41" s="4" t="s">
         <v>41</v>
@@ -1992,10 +1992,10 @@
       </c>
       <c r="F41" s="1"/>
       <c r="G41" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H41" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I41" s="8" t="s">
         <v>2</v>
@@ -2009,7 +2009,7 @@
         <v>45764</v>
       </c>
       <c r="C42" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D42" s="4" t="s">
         <v>6</v>
@@ -2021,10 +2021,10 @@
         <v>301</v>
       </c>
       <c r="G42" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H42" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I42" s="4" t="s">
         <v>2</v>
@@ -2038,7 +2038,7 @@
         <v>45765</v>
       </c>
       <c r="C43" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D43" s="4" t="s">
         <v>4</v>
@@ -2048,10 +2048,10 @@
       </c>
       <c r="F43" s="1"/>
       <c r="G43" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H43" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I43" s="8" t="s">
         <v>2</v>
@@ -2065,7 +2065,7 @@
         <v>45768</v>
       </c>
       <c r="C44" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D44" s="4" t="s">
         <v>4</v>
@@ -2075,10 +2075,10 @@
       </c>
       <c r="F44" s="1"/>
       <c r="G44" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H44" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I44" s="8" t="s">
         <v>2</v>
@@ -2092,7 +2092,7 @@
         <v>45769</v>
       </c>
       <c r="C45" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D45" s="4" t="s">
         <v>4</v>
@@ -2104,10 +2104,10 @@
         <v>315</v>
       </c>
       <c r="G45" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H45" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I45" s="6" t="s">
         <v>2</v>
@@ -2121,7 +2121,7 @@
         <v>45769</v>
       </c>
       <c r="C46" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D46" s="4" t="s">
         <v>5</v>
@@ -2133,10 +2133,10 @@
         <v>315</v>
       </c>
       <c r="G46" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H46" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I46" s="6" t="s">
         <v>2</v>
@@ -2150,7 +2150,7 @@
         <v>45769</v>
       </c>
       <c r="C47" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D47" s="4" t="s">
         <v>3</v>
@@ -2160,10 +2160,10 @@
       </c>
       <c r="F47" s="4"/>
       <c r="G47" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H47" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I47" s="6" t="s">
         <v>2</v>
@@ -2177,7 +2177,7 @@
         <v>45769</v>
       </c>
       <c r="C48" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D48" s="4" t="s">
         <v>3</v>
@@ -2187,10 +2187,10 @@
       </c>
       <c r="F48" s="4"/>
       <c r="G48" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H48" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I48" s="7" t="s">
         <v>2</v>
@@ -2204,7 +2204,7 @@
         <v>45769</v>
       </c>
       <c r="C49" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D49" s="4" t="s">
         <v>4</v>
@@ -2216,10 +2216,10 @@
         <v>329</v>
       </c>
       <c r="G49" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H49" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I49" s="7" t="s">
         <v>2</v>
@@ -2233,7 +2233,7 @@
         <v>45769</v>
       </c>
       <c r="C50" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D50" s="4" t="s">
         <v>4</v>
@@ -2245,10 +2245,10 @@
         <v>330</v>
       </c>
       <c r="G50" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H50" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I50" s="7" t="s">
         <v>2</v>
@@ -2262,7 +2262,7 @@
         <v>45769</v>
       </c>
       <c r="C51" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D51" s="4" t="s">
         <v>4</v>
@@ -2274,10 +2274,10 @@
         <v>331</v>
       </c>
       <c r="G51" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H51" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I51" s="7" t="s">
         <v>2</v>
@@ -2291,7 +2291,7 @@
         <v>45769</v>
       </c>
       <c r="C52" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D52" s="4" t="s">
         <v>4</v>
@@ -2303,10 +2303,10 @@
         <v>332</v>
       </c>
       <c r="G52" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H52" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I52" s="7" t="s">
         <v>2</v>
@@ -2320,7 +2320,7 @@
         <v>45769</v>
       </c>
       <c r="C53" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D53" s="4" t="s">
         <v>4</v>
@@ -2332,10 +2332,10 @@
         <v>333</v>
       </c>
       <c r="G53" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H53" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I53" s="7" t="s">
         <v>2</v>
@@ -2349,7 +2349,7 @@
         <v>45774</v>
       </c>
       <c r="C54" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D54" s="4" t="s">
         <v>4</v>
@@ -2361,10 +2361,10 @@
         <v>325</v>
       </c>
       <c r="G54" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H54" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I54" s="6" t="s">
         <v>2</v>
@@ -2378,7 +2378,7 @@
         <v>45774</v>
       </c>
       <c r="C55" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D55" s="4" t="s">
         <v>5</v>
@@ -2390,10 +2390,10 @@
         <v>325</v>
       </c>
       <c r="G55" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H55" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I55" s="6" t="s">
         <v>2</v>
@@ -2407,7 +2407,7 @@
         <v>45775</v>
       </c>
       <c r="C56" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D56" s="4" t="s">
         <v>4</v>
@@ -2419,10 +2419,10 @@
         <v>327</v>
       </c>
       <c r="G56" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H56" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I56" s="6" t="s">
         <v>2</v>
@@ -2436,7 +2436,7 @@
         <v>45775</v>
       </c>
       <c r="C57" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D57" s="4" t="s">
         <v>5</v>
@@ -2448,10 +2448,10 @@
         <v>327</v>
       </c>
       <c r="G57" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H57" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I57" s="6" t="s">
         <v>2</v>
@@ -2465,22 +2465,22 @@
         <v>45776</v>
       </c>
       <c r="C58" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D58" s="4" t="s">
         <v>6</v>
       </c>
       <c r="E58" s="4" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="F58" s="4" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="G58" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H58" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I58" s="4" t="s">
         <v>2</v>
@@ -2494,7 +2494,7 @@
         <v>45795</v>
       </c>
       <c r="C59" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D59" s="4" t="s">
         <v>3</v>
@@ -2504,10 +2504,10 @@
       </c>
       <c r="F59" s="4"/>
       <c r="G59" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H59" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I59" s="7" t="s">
         <v>36</v>
@@ -2521,7 +2521,7 @@
         <v>45795</v>
       </c>
       <c r="C60" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D60" s="4" t="s">
         <v>4</v>
@@ -2533,10 +2533,10 @@
         <v>337</v>
       </c>
       <c r="G60" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H60" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I60" s="7" t="s">
         <v>36</v>
@@ -2550,7 +2550,7 @@
         <v>45863</v>
       </c>
       <c r="C61" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D61" s="4" t="s">
         <v>41</v>
@@ -2560,10 +2560,10 @@
       </c>
       <c r="F61" s="1"/>
       <c r="G61" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H61" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I61" s="8" t="s">
         <v>2</v>
@@ -2577,7 +2577,7 @@
         <v>45863</v>
       </c>
       <c r="C62" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D62" s="4" t="s">
         <v>4</v>
@@ -2589,10 +2589,10 @@
         <v>336</v>
       </c>
       <c r="G62" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H62" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I62" s="8" t="s">
         <v>2</v>
@@ -2606,7 +2606,7 @@
         <v>45871</v>
       </c>
       <c r="C63" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D63" s="4" t="s">
         <v>3</v>
@@ -2616,10 +2616,10 @@
       </c>
       <c r="F63" s="1"/>
       <c r="G63" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H63" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I63" s="6" t="s">
         <v>17</v>
@@ -2633,7 +2633,7 @@
         <v>45871</v>
       </c>
       <c r="C64" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D64" s="4" t="s">
         <v>4</v>
@@ -2645,10 +2645,10 @@
         <v>342</v>
       </c>
       <c r="G64" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H64" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I64" s="6" t="s">
         <v>17</v>
@@ -2662,7 +2662,7 @@
         <v>45879</v>
       </c>
       <c r="C65" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D65" s="4" t="s">
         <v>3</v>
@@ -2672,10 +2672,10 @@
       </c>
       <c r="F65" s="4"/>
       <c r="G65" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H65" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I65" s="8" t="s">
         <v>2</v>
@@ -2689,7 +2689,7 @@
         <v>45879</v>
       </c>
       <c r="C66" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D66" s="4" t="s">
         <v>4</v>
@@ -2701,10 +2701,10 @@
         <v>341</v>
       </c>
       <c r="G66" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H66" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I66" s="8" t="s">
         <v>2</v>
@@ -2718,7 +2718,7 @@
         <v>45879</v>
       </c>
       <c r="C67" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D67" s="4" t="s">
         <v>4</v>
@@ -2730,10 +2730,10 @@
         <v>341</v>
       </c>
       <c r="G67" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H67" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I67" s="8" t="s">
         <v>2</v>
@@ -2747,7 +2747,7 @@
         <v>45881</v>
       </c>
       <c r="C68" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D68" s="4" t="s">
         <v>3</v>
@@ -2757,10 +2757,10 @@
       </c>
       <c r="F68" s="1"/>
       <c r="G68" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H68" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I68" s="6" t="s">
         <v>19</v>
@@ -2774,7 +2774,7 @@
         <v>45882</v>
       </c>
       <c r="C69" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D69" s="4" t="s">
         <v>3</v>
@@ -2784,10 +2784,10 @@
       </c>
       <c r="F69" s="1"/>
       <c r="G69" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H69" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I69" s="6" t="s">
         <v>10</v>
@@ -2801,7 +2801,7 @@
         <v>45882</v>
       </c>
       <c r="C70" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D70" s="4" t="s">
         <v>3</v>
@@ -2811,10 +2811,10 @@
       </c>
       <c r="F70" s="1"/>
       <c r="G70" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H70" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I70" s="6" t="s">
         <v>10</v>
@@ -2828,7 +2828,7 @@
         <v>45883</v>
       </c>
       <c r="C71" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D71" s="4" t="s">
         <v>3</v>
@@ -2838,10 +2838,10 @@
       </c>
       <c r="F71" s="1"/>
       <c r="G71" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H71" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I71" s="6" t="s">
         <v>19</v>
@@ -2855,7 +2855,7 @@
         <v>45883</v>
       </c>
       <c r="C72" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D72" s="4" t="s">
         <v>4</v>
@@ -2867,10 +2867,10 @@
         <v>343</v>
       </c>
       <c r="G72" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H72" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I72" s="6" t="s">
         <v>19</v>
@@ -2884,7 +2884,7 @@
         <v>45883</v>
       </c>
       <c r="C73" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D73" s="4" t="s">
         <v>5</v>
@@ -2896,10 +2896,10 @@
         <v>343</v>
       </c>
       <c r="G73" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H73" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I73" s="6" t="s">
         <v>19</v>
@@ -2913,7 +2913,7 @@
         <v>45888</v>
       </c>
       <c r="C74" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D74" s="4" t="s">
         <v>3</v>
@@ -2923,10 +2923,10 @@
       </c>
       <c r="F74" s="4"/>
       <c r="G74" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H74" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I74" s="11" t="s">
         <v>2</v>
@@ -2940,7 +2940,7 @@
         <v>45894</v>
       </c>
       <c r="C75" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D75" s="4" t="s">
         <v>3</v>
@@ -2950,10 +2950,10 @@
       </c>
       <c r="F75" s="1"/>
       <c r="G75" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H75" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I75" s="6" t="s">
         <v>19</v>
@@ -2967,7 +2967,7 @@
         <v>45895</v>
       </c>
       <c r="C76" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D76" s="4" t="s">
         <v>6</v>
@@ -2979,10 +2979,10 @@
         <v>315</v>
       </c>
       <c r="G76" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H76" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I76" s="6" t="s">
         <v>2</v>
@@ -2996,7 +2996,7 @@
         <v>45895</v>
       </c>
       <c r="C77" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D77" s="4" t="s">
         <v>3</v>
@@ -3006,10 +3006,10 @@
       </c>
       <c r="F77" s="1"/>
       <c r="G77" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H77" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I77" s="6" t="s">
         <v>10</v>
@@ -3023,7 +3023,7 @@
         <v>45895</v>
       </c>
       <c r="C78" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D78" s="4" t="s">
         <v>3</v>
@@ -3033,10 +3033,10 @@
       </c>
       <c r="F78" s="1"/>
       <c r="G78" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H78" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I78" s="6" t="s">
         <v>10</v>
@@ -3050,7 +3050,7 @@
         <v>45897</v>
       </c>
       <c r="C79" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D79" s="4" t="s">
         <v>3</v>
@@ -3060,10 +3060,10 @@
       </c>
       <c r="F79" s="1"/>
       <c r="G79" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H79" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I79" s="6" t="s">
         <v>19</v>
@@ -3077,7 +3077,7 @@
         <v>45902</v>
       </c>
       <c r="C80" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D80" s="4" t="s">
         <v>5</v>
@@ -3089,10 +3089,10 @@
         <v>337</v>
       </c>
       <c r="G80" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H80" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I80" s="7" t="s">
         <v>36</v>
@@ -3106,7 +3106,7 @@
         <v>45905</v>
       </c>
       <c r="C81" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D81" s="4" t="s">
         <v>3</v>
@@ -3116,10 +3116,10 @@
       </c>
       <c r="F81" s="4"/>
       <c r="G81" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H81" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I81" s="8" t="s">
         <v>2</v>
@@ -3133,7 +3133,7 @@
         <v>45915</v>
       </c>
       <c r="C82" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D82" s="4" t="s">
         <v>3</v>
@@ -3143,10 +3143,10 @@
       </c>
       <c r="F82" s="4"/>
       <c r="G82" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H82" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I82" s="11" t="s">
         <v>2</v>
@@ -3160,7 +3160,7 @@
         <v>45950</v>
       </c>
       <c r="C83" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D83" s="4" t="s">
         <v>5</v>
@@ -3172,10 +3172,10 @@
         <v>342</v>
       </c>
       <c r="G83" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H83" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I83" s="6" t="s">
         <v>17</v>
@@ -3189,7 +3189,7 @@
         <v>45951</v>
       </c>
       <c r="C84" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D84" s="4" t="s">
         <v>5</v>
@@ -3201,10 +3201,10 @@
         <v>336</v>
       </c>
       <c r="G84" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H84" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I84" s="8" t="s">
         <v>2</v>
@@ -3218,7 +3218,7 @@
         <v>45958</v>
       </c>
       <c r="C85" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D85" s="4" t="s">
         <v>5</v>
@@ -3230,10 +3230,10 @@
         <v>340</v>
       </c>
       <c r="G85" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H85" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I85" s="8" t="s">
         <v>2</v>
@@ -3247,7 +3247,7 @@
         <v>45958</v>
       </c>
       <c r="C86" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D86" s="4" t="s">
         <v>5</v>
@@ -3259,10 +3259,10 @@
         <v>341</v>
       </c>
       <c r="G86" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H86" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I86" s="8" t="s">
         <v>2</v>
@@ -3270,13 +3270,13 @@
     </row>
     <row r="87" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B87" s="12">
         <v>45520</v>
       </c>
       <c r="C87" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D87" t="s">
         <v>5</v>
@@ -3288,21 +3288,21 @@
         <v>301</v>
       </c>
       <c r="G87" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="I87" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="88" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B88" s="12">
         <v>45520</v>
       </c>
       <c r="C88" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D88" t="s">
         <v>5</v>
@@ -3314,21 +3314,21 @@
         <v>302</v>
       </c>
       <c r="G88" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="I88" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="89" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B89" s="12">
         <v>45621</v>
       </c>
       <c r="C89" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D89" t="s">
         <v>5</v>
@@ -3340,21 +3340,21 @@
         <v>302</v>
       </c>
       <c r="G89" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="I89" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="90" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B90" s="12">
         <v>45520</v>
       </c>
       <c r="C90" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D90" t="s">
         <v>5</v>
@@ -3366,21 +3366,21 @@
         <v>304</v>
       </c>
       <c r="G90" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="I90" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="91" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B91" s="12">
         <v>45520</v>
       </c>
       <c r="C91" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D91" t="s">
         <v>5</v>
@@ -3392,21 +3392,21 @@
         <v>308</v>
       </c>
       <c r="G91" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="I91" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="92" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B92" s="12">
         <v>45566</v>
       </c>
       <c r="C92" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D92" t="s">
         <v>5</v>
@@ -3418,21 +3418,21 @@
         <v>309</v>
       </c>
       <c r="G92" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="I92" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="93" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B93" s="12">
         <v>45566</v>
       </c>
       <c r="C93" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D93" t="s">
         <v>5</v>
@@ -3444,21 +3444,21 @@
         <v>310</v>
       </c>
       <c r="G93" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="I93" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="94" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B94" s="12">
         <v>45616</v>
       </c>
       <c r="C94" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D94" t="s">
         <v>5</v>
@@ -3470,21 +3470,21 @@
         <v>313</v>
       </c>
       <c r="G94" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="I94" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="95" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B95" s="12">
         <v>45648</v>
       </c>
       <c r="C95" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D95" t="s">
         <v>5</v>
@@ -3496,21 +3496,21 @@
         <v>315</v>
       </c>
       <c r="G95" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="I95" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="96" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B96" s="12">
         <v>45648</v>
       </c>
       <c r="C96" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D96" t="s">
         <v>5</v>
@@ -3522,21 +3522,21 @@
         <v>315</v>
       </c>
       <c r="G96" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="I96" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="97" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B97" s="12">
         <v>45648</v>
       </c>
       <c r="C97" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D97" t="s">
         <v>5</v>
@@ -3548,21 +3548,21 @@
         <v>315</v>
       </c>
       <c r="G97" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="I97" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="98" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B98" s="12">
         <v>45648</v>
       </c>
       <c r="C98" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D98" t="s">
         <v>5</v>
@@ -3574,21 +3574,21 @@
         <v>315</v>
       </c>
       <c r="G98" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="I98" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="99" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A99" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B99" s="12">
         <v>45566</v>
       </c>
       <c r="C99" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D99" t="s">
         <v>5</v>
@@ -3600,21 +3600,21 @@
         <v>317</v>
       </c>
       <c r="G99" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="I99" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="100" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B100" s="12">
         <v>45566</v>
       </c>
       <c r="C100" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D100" t="s">
         <v>5</v>
@@ -3626,21 +3626,21 @@
         <v>317</v>
       </c>
       <c r="G100" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="I100" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="101" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A101" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B101" s="12">
         <v>45755</v>
       </c>
       <c r="C101" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D101" t="s">
         <v>5</v>
@@ -3652,21 +3652,21 @@
         <v>324</v>
       </c>
       <c r="G101" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="I101" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="102" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A102" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B102" s="12">
         <v>45774</v>
       </c>
       <c r="C102" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D102" t="s">
         <v>5</v>
@@ -3678,21 +3678,21 @@
         <v>325</v>
       </c>
       <c r="G102" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="I102" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="103" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A103" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B103" s="12">
         <v>45774</v>
       </c>
       <c r="C103" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D103" t="s">
         <v>5</v>
@@ -3704,21 +3704,21 @@
         <v>325</v>
       </c>
       <c r="G103" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="I103" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="104" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A104" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B104" s="12">
         <v>45774</v>
       </c>
       <c r="C104" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D104" t="s">
         <v>5</v>
@@ -3730,21 +3730,21 @@
         <v>325</v>
       </c>
       <c r="G104" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="I104" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="105" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A105" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B105" s="12">
         <v>45774</v>
       </c>
       <c r="C105" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D105" t="s">
         <v>5</v>
@@ -3756,21 +3756,21 @@
         <v>325</v>
       </c>
       <c r="G105" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="I105" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="106" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A106" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B106" s="12">
         <v>45951</v>
       </c>
       <c r="C106" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D106" t="s">
         <v>5</v>
@@ -3782,21 +3782,21 @@
         <v>336</v>
       </c>
       <c r="G106" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="I106" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="107" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A107" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="B107" s="12">
         <v>45608</v>
       </c>
       <c r="C107" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D107" t="s">
         <v>6</v>
@@ -3808,21 +3808,21 @@
         <v>301</v>
       </c>
       <c r="G107" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="I107" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="108" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A108" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B108" s="12">
         <v>45621</v>
       </c>
       <c r="C108" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D108" t="s">
         <v>6</v>
@@ -3834,21 +3834,21 @@
         <v>302</v>
       </c>
       <c r="G108" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="I108" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="109" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A109" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B109" s="12">
         <v>45566</v>
       </c>
       <c r="C109" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D109" t="s">
         <v>6</v>
@@ -3860,21 +3860,21 @@
         <v>309</v>
       </c>
       <c r="G109" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="I109" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="110" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A110" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B110" s="12">
         <v>45566</v>
       </c>
       <c r="C110" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D110" t="s">
         <v>6</v>
@@ -3886,21 +3886,21 @@
         <v>310</v>
       </c>
       <c r="G110" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="I110" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="111" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A111" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B111" s="12">
         <v>45616</v>
       </c>
       <c r="C111" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D111" t="s">
         <v>6</v>
@@ -3912,21 +3912,21 @@
         <v>314</v>
       </c>
       <c r="G111" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="I111" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="112" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A112" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="B112" s="12">
         <v>45713</v>
       </c>
       <c r="C112" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D112" t="s">
         <v>6</v>
@@ -3938,21 +3938,21 @@
         <v>316</v>
       </c>
       <c r="G112" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="I112" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="113" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A113" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B113" s="12">
         <v>45566</v>
       </c>
       <c r="C113" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D113" t="s">
         <v>6</v>
@@ -3964,21 +3964,21 @@
         <v>318</v>
       </c>
       <c r="G113" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="I113" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="114" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A114" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B114" s="12">
         <v>45713</v>
       </c>
       <c r="C114" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D114" t="s">
         <v>6</v>
@@ -3990,21 +3990,21 @@
         <v>320</v>
       </c>
       <c r="G114" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="I114" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="115" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A115" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="B115" s="12">
         <v>45599</v>
       </c>
       <c r="C115" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D115" t="s">
         <v>6</v>
@@ -4016,24 +4016,24 @@
         <v>321</v>
       </c>
       <c r="G115" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="I115" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="116" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A116" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="B116" s="12">
         <v>45520</v>
       </c>
       <c r="C116" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D116" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="E116" t="s">
         <v>1</v>
@@ -4042,27 +4042,27 @@
         <v>301</v>
       </c>
       <c r="G116" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H116" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I116" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
     </row>
     <row r="117" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A117" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="B117" s="12">
         <v>45520</v>
       </c>
       <c r="C117" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D117" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="E117" t="s">
         <v>1</v>
@@ -4071,24 +4071,24 @@
         <v>302</v>
       </c>
       <c r="G117" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H117" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I117" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
     </row>
     <row r="118" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A118" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="B118" s="12">
         <v>45620</v>
       </c>
       <c r="C118" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D118" t="s">
         <v>5</v>
@@ -4100,24 +4100,24 @@
         <v>301</v>
       </c>
       <c r="G118" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H118" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I118" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
     </row>
     <row r="119" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A119" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="B119" s="12">
         <v>45621</v>
       </c>
       <c r="C119" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D119" t="s">
         <v>5</v>
@@ -4129,24 +4129,24 @@
         <v>302</v>
       </c>
       <c r="G119" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H119" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I119" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
     </row>
     <row r="120" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A120" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="B120" s="12">
         <v>45764</v>
       </c>
       <c r="C120" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D120" t="s">
         <v>6</v>
@@ -4158,24 +4158,24 @@
         <v>301</v>
       </c>
       <c r="G120" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H120" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I120" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
     </row>
     <row r="121" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A121" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="B121" s="12">
         <v>45719</v>
       </c>
       <c r="C121" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D121" t="s">
         <v>6</v>
@@ -4187,53 +4187,53 @@
         <v>302</v>
       </c>
       <c r="G121" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H121" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I121" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
     </row>
     <row r="122" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A122" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B122" s="12">
         <v>45938</v>
       </c>
       <c r="C122" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D122" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="H122" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="I122" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
     </row>
     <row r="123" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A123" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="B123" s="12">
         <v>45712</v>
       </c>
       <c r="C123" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D123" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="G123" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="I123" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="124" spans="1:9" x14ac:dyDescent="0.2">

</xml_diff>